<commit_message>
auto: CV Arago (HRIS & AI Tech Pre-Sales) + maj tableur
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -3931,7 +3931,11 @@
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
-      <c r="B46" s="40" t="n"/>
+      <c r="B46" s="40" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
       <c r="C46" s="40" t="n"/>
       <c r="D46" s="5" t="inlineStr">
         <is>
@@ -3977,7 +3981,7 @@
       </c>
       <c r="N46" s="40" t="inlineStr">
         <is>
-          <t>CV_GaetanFRANCOIS_CSM_EN.html</t>
+          <t>Resume_GaetanFRANCOIS_Arago.pdf</t>
         </is>
       </c>
       <c r="O46" s="40" t="inlineStr">

</xml_diff>

<commit_message>
auto: Arago HRIS & AI Tech Pre-Sales marqué Postulé
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -1388,21 +1388,25 @@
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Postulé</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="n"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Group HRIS Manager</t>
+          <t>HRIS &amp; AI Tech Pre-Sales Specialist</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>CLM Search (groupe industriel mondial)</t>
+          <t>Arago Consulting</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>SmartRecruiters</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -1412,41 +1416,42 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Paris ou Bordeaux</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Hybride</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>n.c.</t>
-        </is>
-      </c>
+          <t>Partiel (déplacements clients)</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Groupe industriel 40+ pays, 170K salariés, 30Mds€ — SF expertise non negotiable (Comp/Recruiting/Reporting) — évolution HRIS Director — FIT PARFAIT (L'Oréal 40+ pays)</t>
+          <t>Arago = 1er partenaire européen SAP SuccessFactors. Croisement parfait pre-sales IA+SIRH : 14 ans SAP, 40 pays L'Oréal, usage quotidien IA générative, profil face-client senior. Bordeaux = 2h d'Anglet. Lien : jobs.smartrecruiters.com/Arago/744000139094386 Postulé le 04/08/2026 (CV Resume_GaetanFRANCOIS_Arago.pdf + message hiring team).</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/4415288591</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Resume_GaetanFRANCOIS_SIRH_EN.pdf</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>95 K€</t>
-        </is>
-      </c>
-      <c r="Q7" s="42" t="n"/>
+          <t>https://jobs.smartrecruiters.com/Arago/744000139094386-hris-ai-tech-pre-sales-specialist</t>
+        </is>
+      </c>
+      <c r="N7" s="40" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Arago.pdf</t>
+        </is>
+      </c>
+      <c r="O7" s="40" t="inlineStr">
+        <is>
+          <t>90-110K€</t>
+        </is>
+      </c>
+      <c r="P7" s="40" t="n"/>
+      <c r="Q7" s="42" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="8" hidden="1" ht="40" customHeight="1">
       <c r="A8" s="78" t="inlineStr">
@@ -1458,17 +1463,17 @@
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Senior Manager Conseil Talent Management F/H</t>
+          <t>Group HRIS Manager</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>HRConseil</t>
+          <t>CLM Search (groupe industriel mondial)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>SmartRecruiters</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -1483,43 +1488,39 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Hybride (3j/sem)</t>
+          <t>Hybride</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>75 000 - 85 000 € + 8 000 € bonus</t>
+          <t>n.c.</t>
         </is>
       </c>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Cabinet conseil SIRH (Workday, SF, Oracle HCM). 15+ ans requis, maîtrise SF, face client, avant-vente, management consultants. Salaire dans la cible haute. Fit parfait avec le profil Gaëtan (15 ans, SAP/SF, L'Oréal, avant-vente).</t>
+          <t>Groupe industriel 40+ pays, 170K salariés, 30Mds€ — SF expertise non negotiable (Comp/Recruiting/Reporting) — évolution HRIS Director — FIT PARFAIT (L'Oréal 40+ pays)</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/HRConseil1/744000100293238-senior-manager-conseil-talent-management-f-h-cdi</t>
+          <t>https://fr.linkedin.com/jobs/view/4415288591</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_SIRH.pdf</t>
+          <t>Resume_GaetanFRANCOIS_SIRH_EN.pdf</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>82 K€</t>
-        </is>
-      </c>
-      <c r="Q8" s="42" t="inlineStr">
-        <is>
-          <t>27/05/2026</t>
-        </is>
-      </c>
+          <t>95 K€</t>
+        </is>
+      </c>
+      <c r="Q8" s="42" t="n"/>
     </row>
     <row r="9" hidden="1" ht="40" customHeight="1">
-      <c r="A9" s="77" t="inlineStr">
+      <c r="A9" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
@@ -1528,17 +1529,17 @@
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Senior Principal Success Manager</t>
+          <t>Senior Manager Conseil Talent Management F/H</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>HRConseil</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Salesforce Careers</t>
+          <t>SmartRecruiters</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1553,29 +1554,38 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Hybride</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="n"/>
+          <t>Hybride (3j/sem)</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>75 000 - 85 000 € + 8 000 € bonus</t>
+        </is>
+      </c>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Niveau CSM le plus élevé chez Salesforce France, profil 15 ans exact, posté 23/03/2026</t>
+          <t>Cabinet conseil SIRH (Workday, SF, Oracle HCM). 15+ ans requis, maîtrise SF, face client, avant-vente, management consultants. Salaire dans la cible haute. Fit parfait avec le profil Gaëtan (15 ans, SAP/SF, L'Oréal, avant-vente).</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>https://careers.salesforce.com/en/jobs/jr330883/senior-principal-success-manager/</t>
+          <t>https://jobs.smartrecruiters.com/HRConseil1/744000100293238-senior-manager-conseil-talent-management-f-h-cdi</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS.pdf</t>
+          <t>Resume_GaetanFRANCOIS_SIRH.pdf</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>82 K€</t>
         </is>
       </c>
       <c r="Q9" s="42" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
     </row>
@@ -1589,17 +1599,17 @@
       <c r="C10" s="6" t="n"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Consultant SAP SuccessFactors H/F</t>
+          <t>Senior Principal Success Manager</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>HR Path</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>HR Path Careers</t>
+          <t>Salesforce Careers</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -1609,7 +1619,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Paris La Défense</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -1621,27 +1631,27 @@
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Cabinet SIRH majeur, projets SF internationaux, 2 ans mini SF — profil L'Oréal 40 pays en cible directe</t>
+          <t>Niveau CSM le plus élevé chez Salesforce France, profil 15 ans exact, posté 23/03/2026</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.hr-path.com/job/Paris-La-D%C3%A9fense-Cedex-Consultant-SAP-SuccessFactors-(HF)-75-92042/818651901/</t>
+          <t>https://careers.salesforce.com/en/jobs/jr330883/senior-principal-success-manager/</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_SIRH.pdf</t>
+          <t>Resume_GaetanFRANCOIS.pdf</t>
         </is>
       </c>
       <c r="Q10" s="42" t="inlineStr">
         <is>
-          <t>17/06/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
     </row>
     <row r="11" hidden="1" ht="40" customHeight="1">
-      <c r="A11" s="78" t="inlineStr">
+      <c r="A11" s="77" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
@@ -1650,52 +1660,49 @@
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Directeur de Programme SIRH Senior H/F</t>
+          <t>Consultant SAP SuccessFactors H/F</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>LeHibou (client grand groupe)</t>
+          <t>HR Path</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>free-work.com</t>
+          <t>HR Path Careers</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Freelance</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Paris La Défense</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>650-780 €/j</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>18 mois (démarrage août 2026)</t>
-        </is>
-      </c>
+          <t>Hybride</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Pilotage transformation RH grand groupe international bout en bout. 15 ans requis, SAP SF/TalentSoft/Workday. TJM dans cible haute, durée longue. Profil parfait.</t>
+          <t>Cabinet SIRH majeur, projets SF internationaux, 2 ans mini SF — profil L'Oréal 40 pays en cible directe</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>https://www.free-work.com/fr/tech-it/job-mission/administrateur-applicatif-erp-crm-sirh/mission-freelance-directeur-de-programme-sirh-senior-h-f</t>
+          <t>https://jobs.hr-path.com/job/Paris-La-D%C3%A9fense-Cedex-Consultant-SAP-SuccessFactors-(HF)-75-92042/818651901/</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_SIRH.pdf</t>
         </is>
       </c>
       <c r="Q11" s="42" t="inlineStr">
@@ -1705,7 +1712,7 @@
       </c>
     </row>
     <row r="12" hidden="1" ht="40" customHeight="1">
-      <c r="A12" s="77" t="inlineStr">
+      <c r="A12" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
@@ -1714,124 +1721,121 @@
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
+          <t>Directeur de Programme SIRH Senior H/F</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>LeHibou (client grand groupe)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>free-work.com</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>650-780 €/j</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>18 mois (démarrage août 2026)</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage transformation RH grand groupe international bout en bout. 15 ans requis, SAP SF/TalentSoft/Workday. TJM dans cible haute, durée longue. Profil parfait.</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.free-work.com/fr/tech-it/job-mission/administrateur-applicatif-erp-crm-sirh/mission-freelance-directeur-de-programme-sirh-senior-h-f</t>
+        </is>
+      </c>
+      <c r="Q12" s="42" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" hidden="1" ht="40" customHeight="1">
+      <c r="A13" s="77" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
           <t>Consultant(e) SIRH – Audit SIRH Grand Groupe</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Client grand groupe (via Le Club des RH)</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>leclubdesrh.fr</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Freelance</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Partiel (2j/sem)</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>900 €/j</t>
         </is>
       </c>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="5" t="inlineStr">
         <is>
           <t>TJM 900€/j. Audit SIRH grand groupe, 2j/sem Paris. Mission visible uniquement après inscription sur app.leclubdesrh.fr (rejoindre la communauté via airtable.com/appqNConNIfeCCjB8/shrhxbRraMvUqda2C).</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M13" s="5" t="inlineStr">
         <is>
           <t>https://app.leclubdesrh.fr/</t>
-        </is>
-      </c>
-      <c r="N12" s="40" t="n"/>
-      <c r="O12" s="40" t="n"/>
-      <c r="P12" s="40" t="n"/>
-      <c r="Q12" s="42" t="n"/>
-    </row>
-    <row r="13" hidden="1" ht="40" customHeight="1">
-      <c r="A13" s="78" t="inlineStr">
-        <is>
-          <t>⭐⭐⭐⭐⭐</t>
-        </is>
-      </c>
-      <c r="B13" s="40" t="n"/>
-      <c r="C13" s="40" t="n"/>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Directeur de Programme SIRH Senior H/F</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>LeHibou (client grand groupe)</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>free-work.com</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Freelance</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>Partiel</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>650-780 €/j</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>18 mois (démarrage août 2026)</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>Pilotage transformation RH grand groupe international bout en bout. 15 ans requis, SAP SF/Workday. TJM dans cible haute, durée longue.</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
-        <is>
-          <t>https://www.free-work.com/fr/tech-it/job-mission/administrateur-applicatif-erp-crm-sirh/mission-freelance-directeur-de-programme-sirh-senior-h-f</t>
         </is>
       </c>
       <c r="N13" s="40" t="n"/>
       <c r="O13" s="40" t="n"/>
       <c r="P13" s="40" t="n"/>
-      <c r="Q13" s="42" t="inlineStr">
-        <is>
-          <t>17/06/2026</t>
-        </is>
-      </c>
+      <c r="Q13" s="42" t="n"/>
     </row>
     <row r="14" hidden="1" ht="40" customHeight="1">
-      <c r="A14" s="77" t="inlineStr">
+      <c r="A14" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
@@ -1840,73 +1844,65 @@
       <c r="C14" s="40" t="n"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Data Migration SAP SuccessFactors Consultant (24 mois)</t>
+          <t>Directeur de Programme SIRH Senior H/F</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>n.c. (via Freelance-Informatique)</t>
+          <t>LeHibou (client grand groupe)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Freelance-Informatique</t>
+          <t>free-work.com</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Mission</t>
+          <t>Freelance</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Clichy (92)</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Hybride</t>
+          <t>Partiel</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>N/C</t>
+          <t>650-780 €/j</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>24 mois (démarrage ASAP)</t>
+          <t>18 mois (démarrage août 2026)</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Spécialité migration données SAP SuccessFactors. Profil Gaëtan : migration SAP HR → SF sur L'Oréal 40+ pays = différenciant majeur. Mission longue et très alignée.</t>
+          <t>Pilotage transformation RH grand groupe international bout en bout. 15 ans requis, SAP SF/Workday. TJM dans cible haute, durée longue.</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>https://www.freelance-informatique.fr/cv-mission-consultant-sap-successfactors-freelance-f11256</t>
-        </is>
-      </c>
-      <c r="N14" s="40" t="inlineStr">
-        <is>
-          <t>Resume_GaetanFRANCOIS_SIRH</t>
-        </is>
-      </c>
-      <c r="O14" s="40" t="inlineStr">
-        <is>
-          <t>650-750€/j</t>
-        </is>
-      </c>
+          <t>https://www.free-work.com/fr/tech-it/job-mission/administrateur-applicatif-erp-crm-sirh/mission-freelance-directeur-de-programme-sirh-senior-h-f</t>
+        </is>
+      </c>
+      <c r="N14" s="40" t="n"/>
+      <c r="O14" s="40" t="n"/>
       <c r="P14" s="40" t="n"/>
       <c r="Q14" s="42" t="inlineStr">
         <is>
-          <t>07/07/2026</t>
+          <t>17/06/2026</t>
         </is>
       </c>
     </row>
     <row r="15" hidden="1" ht="40" customHeight="1">
-      <c r="A15" s="78" t="inlineStr">
+      <c r="A15" s="77" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
@@ -1915,65 +1911,73 @@
       <c r="C15" s="40" t="n"/>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>HR Tech Run Lead</t>
+          <t>Data Migration SAP SuccessFactors Consultant (24 mois)</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>L'Oréal</t>
+          <t>n.c. (via Freelance-Informatique)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Freelance-Informatique</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>Mission</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Biarritz</t>
+          <t>Clichy (92)</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Hybride (3j bureau / 2j remote)</t>
+          <t>Hybride</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>nc</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="n"/>
+          <t>N/C</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>24 mois (démarrage ASAP)</t>
+        </is>
+      </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>EXCEPTIONNEL : Biarritz + 10 ans L'Oréal SAP HCM/SF dans le profil — 10+ ans HRIS requis — posté il y a 5 jours</t>
+          <t>Spécialité migration données SAP SuccessFactors. Profil Gaëtan : migration SAP HR → SF sur L'Oréal 40+ pays = différenciant majeur. Mission longue et très alignée.</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/hr-tech-run-lead-at-l-or%C3%A9al-4435534808</t>
+          <t>https://www.freelance-informatique.fr/cv-mission-consultant-sap-successfactors-freelance-f11256</t>
         </is>
       </c>
       <c r="N15" s="40" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_SIRH.html</t>
+          <t>Resume_GaetanFRANCOIS_SIRH</t>
         </is>
       </c>
       <c r="O15" s="40" t="inlineStr">
         <is>
-          <t>90-110K€</t>
+          <t>650-750€/j</t>
         </is>
       </c>
       <c r="P15" s="40" t="n"/>
-      <c r="Q15" s="42" t="n"/>
+      <c r="Q15" s="42" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="16" hidden="1" ht="40" customHeight="1">
-      <c r="A16" s="77" t="inlineStr">
+      <c r="A16" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
@@ -1982,12 +1986,12 @@
       <c r="C16" s="40" t="n"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Senior AMOA Talent Consultant M/F</t>
+          <t>HR Tech Run Lead</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>MP People</t>
+          <t>L'Oréal</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -2002,33 +2006,45 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Biarritz</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="n"/>
+          <t>Hybride (3j bureau / 2j remote)</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>nc</t>
+        </is>
+      </c>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>AMOA Talent senior = profil exact ; posté hier</t>
+          <t>EXCEPTIONNEL : Biarritz + 10 ans L'Oréal SAP HCM/SF dans le profil — 10+ ans HRIS requis — posté il y a 5 jours</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/senior-amoa-talent-consultant-m-f-at-mp-people-4437133991</t>
-        </is>
-      </c>
-      <c r="N16" s="40" t="n"/>
-      <c r="O16" s="40" t="n"/>
+          <t>https://fr.linkedin.com/jobs/view/hr-tech-run-lead-at-l-or%C3%A9al-4435534808</t>
+        </is>
+      </c>
+      <c r="N16" s="40" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_SIRH.html</t>
+        </is>
+      </c>
+      <c r="O16" s="40" t="inlineStr">
+        <is>
+          <t>90-110K€</t>
+        </is>
+      </c>
       <c r="P16" s="40" t="n"/>
       <c r="Q16" s="42" t="n"/>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="78" t="inlineStr">
+      <c r="A17" s="77" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
@@ -2037,7 +2053,7 @@
       <c r="C17" s="40" t="n"/>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Consultant Senior AMOA Talent H/F</t>
+          <t>Senior AMOA Talent Consultant M/F</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -2069,18 +2085,18 @@
       <c r="K17" s="6" t="n"/>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>Variante Senior AMOA Talent ; posté hier</t>
+          <t>AMOA Talent senior = profil exact ; posté hier</t>
         </is>
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/consultant-senior-amoa-talent-h-f-at-mp-people-4437143555</t>
+          <t>https://fr.linkedin.com/jobs/view/senior-amoa-talent-consultant-m-f-at-mp-people-4437133991</t>
         </is>
       </c>
       <c r="N17" s="40" t="n"/>
       <c r="O17" s="40" t="n"/>
       <c r="P17" s="40" t="n"/>
-      <c r="Q17" s="40" t="n"/>
+      <c r="Q17" s="42" t="n"/>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="78" t="inlineStr">
@@ -2092,7 +2108,7 @@
       <c r="C18" s="40" t="n"/>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Manager AMOA Talent M/F</t>
+          <t>Consultant Senior AMOA Talent H/F</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -2124,12 +2140,12 @@
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>Manager AMOA Talent ; 3 postes MP People simultanés = cabinet en forte croissance</t>
+          <t>Variante Senior AMOA Talent ; posté hier</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/manager-amoa-talent-m-f-at-mp-people-4437146495</t>
+          <t>https://fr.linkedin.com/jobs/view/consultant-senior-amoa-talent-h-f-at-mp-people-4437143555</t>
         </is>
       </c>
       <c r="N18" s="40" t="n"/>
@@ -2138,75 +2154,59 @@
       <c r="Q18" s="40" t="n"/>
     </row>
     <row r="19" hidden="1" ht="40" customHeight="1">
-      <c r="A19" s="83" t="inlineStr">
+      <c r="A19" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
       <c r="B19" s="40" t="n"/>
       <c r="C19" s="40" t="n"/>
-      <c r="D19" s="40" t="inlineStr">
-        <is>
-          <t>Directeur de Programme SIRH Senior H/F</t>
-        </is>
-      </c>
-      <c r="E19" s="40" t="inlineStr">
-        <is>
-          <t>LeHibou</t>
-        </is>
-      </c>
-      <c r="F19" s="40" t="inlineStr">
-        <is>
-          <t>free-work</t>
-        </is>
-      </c>
-      <c r="G19" s="40" t="inlineStr">
-        <is>
-          <t>Mission freelance</t>
-        </is>
-      </c>
-      <c r="H19" s="40" t="inlineStr">
-        <is>
-          <t>Paris (75)</t>
-        </is>
-      </c>
-      <c r="I19" s="40" t="inlineStr">
-        <is>
-          <t>N/C</t>
-        </is>
-      </c>
-      <c r="J19" s="40" t="inlineStr">
-        <is>
-          <t>650-780€/j</t>
-        </is>
-      </c>
-      <c r="K19" s="40" t="inlineStr">
-        <is>
-          <t>18 mois</t>
-        </is>
-      </c>
-      <c r="L19" s="40" t="inlineStr">
-        <is>
-          <t>Programme RH grand groupe, SAP SF + PowerBI, fort fit ; 17/06/2026</t>
-        </is>
-      </c>
-      <c r="M19" s="40" t="inlineStr">
-        <is>
-          <t>https://www.free-work.com/fr/tech-it/job-mission/administrateur-applicatif-erp-crm-sirh/mission-freelance-directeur-de-programme-sirh-senior-h-f</t>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Manager AMOA Talent M/F</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>MP People</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Manager AMOA Talent ; 3 postes MP People simultanés = cabinet en forte croissance</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/manager-amoa-talent-m-f-at-mp-people-4437146495</t>
         </is>
       </c>
       <c r="N19" s="40" t="n"/>
       <c r="O19" s="40" t="n"/>
-      <c r="P19" s="40" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="Q19" s="40" t="inlineStr">
-        <is>
-          <t>17/06/2026</t>
-        </is>
-      </c>
+      <c r="P19" s="40" t="n"/>
+      <c r="Q19" s="40" t="n"/>
     </row>
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="83" t="inlineStr">
@@ -2218,52 +2218,52 @@
       <c r="C20" s="40" t="n"/>
       <c r="D20" s="40" t="inlineStr">
         <is>
-          <t>SAP Project Manager / Trainer</t>
+          <t>Directeur de Programme SIRH Senior H/F</t>
         </is>
       </c>
       <c r="E20" s="40" t="inlineStr">
         <is>
-          <t>N/C (via eursap.eu)</t>
+          <t>LeHibou</t>
         </is>
       </c>
       <c r="F20" s="40" t="inlineStr">
         <is>
-          <t>eursap.eu</t>
+          <t>free-work</t>
         </is>
       </c>
       <c r="G20" s="40" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>Mission freelance</t>
         </is>
       </c>
       <c r="H20" s="40" t="inlineStr">
         <is>
-          <t>100% Remote</t>
+          <t>Paris (75)</t>
         </is>
       </c>
       <c r="I20" s="40" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>N/C</t>
         </is>
       </c>
       <c r="J20" s="40" t="inlineStr">
         <is>
-          <t>80-156k€/an + equity</t>
+          <t>650-780€/j</t>
         </is>
       </c>
       <c r="K20" s="40" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>18 mois</t>
         </is>
       </c>
       <c r="L20" s="40" t="inlineStr">
         <is>
-          <t>SAP PM + formateur, full remote, fourchette haute, démarrage août 2026 ; ref 34811</t>
+          <t>Programme RH grand groupe, SAP SF + PowerBI, fort fit ; 17/06/2026</t>
         </is>
       </c>
       <c r="M20" s="40" t="inlineStr">
         <is>
-          <t>https://eursap.eu/sap-jobs/france/</t>
+          <t>https://www.free-work.com/fr/tech-it/job-mission/administrateur-applicatif-erp-crm-sirh/mission-freelance-directeur-de-programme-sirh-senior-h-f</t>
         </is>
       </c>
       <c r="N20" s="40" t="n"/>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="Q20" s="40" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>17/06/2026</t>
         </is>
       </c>
     </row>
@@ -2289,27 +2289,27 @@
       <c r="C21" s="40" t="n"/>
       <c r="D21" s="40" t="inlineStr">
         <is>
-          <t>Chef de Projet Fonctionnel SIRH 100% Remote</t>
+          <t>SAP Project Manager / Trainer</t>
         </is>
       </c>
       <c r="E21" s="40" t="inlineStr">
         <is>
-          <t>N/C</t>
+          <t>N/C (via eursap.eu)</t>
         </is>
       </c>
       <c r="F21" s="40" t="inlineStr">
         <is>
-          <t>freelance-informatique.fr</t>
+          <t>eursap.eu</t>
         </is>
       </c>
       <c r="G21" s="40" t="inlineStr">
         <is>
-          <t>Mission freelance</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="H21" s="40" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>100% Remote</t>
         </is>
       </c>
       <c r="I21" s="40" t="inlineStr">
@@ -2319,34 +2319,34 @@
       </c>
       <c r="J21" s="40" t="inlineStr">
         <is>
-          <t>N/C</t>
+          <t>80-156k€/an + equity</t>
         </is>
       </c>
       <c r="K21" s="40" t="inlineStr">
         <is>
-          <t>6 mois</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="L21" s="40" t="inlineStr">
         <is>
-          <t>Full remote, ASAP ; freelance-info ; 10/07/2026</t>
+          <t>SAP PM + formateur, full remote, fourchette haute, démarrage août 2026 ; ref 34811</t>
         </is>
       </c>
       <c r="M21" s="40" t="inlineStr">
         <is>
-          <t>https://www.freelance-informatique.fr/chef-de-projet-sirh-freelance-n112</t>
+          <t>https://eursap.eu/sap-jobs/france/</t>
         </is>
       </c>
       <c r="N21" s="40" t="n"/>
       <c r="O21" s="40" t="n"/>
       <c r="P21" s="40" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>09/07/2026</t>
         </is>
       </c>
       <c r="Q21" s="40" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
     </row>
@@ -2360,32 +2360,32 @@
       <c r="C22" s="40" t="n"/>
       <c r="D22" s="40" t="inlineStr">
         <is>
-          <t>HRIS Project Manager</t>
+          <t>Chef de Projet Fonctionnel SIRH 100% Remote</t>
         </is>
       </c>
       <c r="E22" s="40" t="inlineStr">
         <is>
-          <t>Next Ventures</t>
+          <t>N/C</t>
         </is>
       </c>
       <c r="F22" s="40" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>freelance-informatique.fr</t>
         </is>
       </c>
       <c r="G22" s="40" t="inlineStr">
         <is>
-          <t>Contrat 6 mois</t>
+          <t>Mission freelance</t>
         </is>
       </c>
       <c r="H22" s="40" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="I22" s="40" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="J22" s="40" t="inlineStr">
@@ -2400,12 +2400,12 @@
       </c>
       <c r="L22" s="40" t="inlineStr">
         <is>
-          <t>SAP SF + ServiceNow, secteur financier, fort fit ; 03/07/2026</t>
-        </is>
-      </c>
-      <c r="M22" s="91" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/hris-sirh-project-manager-at-next-ventures-4433811211</t>
+          <t>Full remote, ASAP ; freelance-info ; 10/07/2026</t>
+        </is>
+      </c>
+      <c r="M22" s="40" t="inlineStr">
+        <is>
+          <t>https://www.freelance-informatique.fr/chef-de-projet-sirh-freelance-n112</t>
         </is>
       </c>
       <c r="N22" s="40" t="n"/>
@@ -2417,87 +2417,83 @@
       </c>
       <c r="Q22" s="40" t="inlineStr">
         <is>
-          <t>03/07/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
     </row>
     <row r="23" hidden="1" ht="40" customHeight="1">
-      <c r="A23" s="77" t="inlineStr">
+      <c r="A23" s="83" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
       <c r="B23" s="40" t="n"/>
       <c r="C23" s="40" t="n"/>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Global Tech HR Domain Manager F/M/X</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Sephora</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>Neuilly-sur-Seine</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>À clarifier</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>À négocier (viser 90-110K€)</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="L23" s="5" t="inlineStr">
-        <is>
-          <t>Supervision déploiement RH/SAP, coordination équipes internes + partenaires ext = profil DPO exact. LVMH group. Publié 13/07/2026. Proche profil L'Oréal HR Domain.</t>
-        </is>
-      </c>
-      <c r="M23" s="5" t="inlineStr">
-        <is>
-          <t>https://fr.indeed.com/q-consultant-sap-successfactors-emplois.html</t>
-        </is>
-      </c>
-      <c r="N23" s="40" t="inlineStr">
-        <is>
-          <t>Resume_GaetanFRANCOIS_SIRH_EN.pdf</t>
-        </is>
-      </c>
-      <c r="O23" s="40" t="inlineStr">
-        <is>
-          <t>90-110K€</t>
-        </is>
-      </c>
-      <c r="P23" s="40" t="n"/>
-      <c r="Q23" s="42" t="inlineStr">
-        <is>
-          <t>18/06/2026</t>
+      <c r="D23" s="40" t="inlineStr">
+        <is>
+          <t>HRIS Project Manager</t>
+        </is>
+      </c>
+      <c r="E23" s="40" t="inlineStr">
+        <is>
+          <t>Next Ventures</t>
+        </is>
+      </c>
+      <c r="F23" s="40" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G23" s="40" t="inlineStr">
+        <is>
+          <t>Contrat 6 mois</t>
+        </is>
+      </c>
+      <c r="H23" s="40" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I23" s="40" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="J23" s="40" t="inlineStr">
+        <is>
+          <t>N/C</t>
+        </is>
+      </c>
+      <c r="K23" s="40" t="inlineStr">
+        <is>
+          <t>6 mois</t>
+        </is>
+      </c>
+      <c r="L23" s="40" t="inlineStr">
+        <is>
+          <t>SAP SF + ServiceNow, secteur financier, fort fit ; 03/07/2026</t>
+        </is>
+      </c>
+      <c r="M23" s="91" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/hris-sirh-project-manager-at-next-ventures-4433811211</t>
+        </is>
+      </c>
+      <c r="N23" s="40" t="n"/>
+      <c r="O23" s="40" t="n"/>
+      <c r="P23" s="40" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="Q23" s="40" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
         </is>
       </c>
     </row>
     <row r="24" hidden="1" ht="40" customHeight="1">
-      <c r="A24" s="78" t="inlineStr">
+      <c r="A24" s="77" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
@@ -2506,12 +2502,12 @@
       <c r="C24" s="40" t="n"/>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>HR Domain Manager</t>
+          <t>Global Tech HR Domain Manager F/M/X</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Parfums Christian Dior</t>
+          <t>Sephora</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -2546,7 +2542,7 @@
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>LVMH. Coordination équipes internes, consultants externes et équipes dev Finance &amp; HR. Fit direct 10 ans L'Oréal = same environment. Publié 13/07/2026.</t>
+          <t>Supervision déploiement RH/SAP, coordination équipes internes + partenaires ext = profil DPO exact. LVMH group. Publié 13/07/2026. Proche profil L'Oréal HR Domain.</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
@@ -2565,33 +2561,33 @@
         </is>
       </c>
       <c r="P24" s="40" t="n"/>
-      <c r="Q24" s="42" t="n"/>
+      <c r="Q24" s="42" t="inlineStr">
+        <is>
+          <t>18/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="25" hidden="1" ht="40" customHeight="1">
-      <c r="A25" s="77" t="inlineStr">
+      <c r="A25" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
-      <c r="B25" s="40" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
+      <c r="B25" s="40" t="n"/>
       <c r="C25" s="40" t="n"/>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Responsable SIRH F/H</t>
+          <t>HR Domain Manager</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>KPMG France</t>
+          <t>Parfums Christian Dior</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Welcome to the Jungle / emplois.kpmg.fr</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -2601,42 +2597,46 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Courbevoie / La Défense</t>
+          <t>Neuilly-sur-Seine</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>À clarifier</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>Non affiché</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="n"/>
+          <t>À négocier (viser 90-110K€)</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>KPMG migration PeopleSoft → SAP SuccessFactors. Responsable SIRH = manager équipe + pilote roadmap. Requis 10 ans+ SIRH + team management + Core HR. Parfait fit Gaëtan (14 ans SAP + L'Oréal 40 pays). Démarrage mars 2026.</t>
+          <t>LVMH. Coordination équipes internes, consultants externes et équipes dev Finance &amp; HR. Fit direct 10 ans L'Oréal = same environment. Publié 13/07/2026.</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/fr/companies/kpmg-france/jobs/responsable-sirh-f-h_courbevoie</t>
-        </is>
-      </c>
-      <c r="N25" s="40" t="n"/>
+          <t>https://fr.indeed.com/q-consultant-sap-successfactors-emplois.html</t>
+        </is>
+      </c>
+      <c r="N25" s="40" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_SIRH_EN.pdf</t>
+        </is>
+      </c>
       <c r="O25" s="40" t="inlineStr">
         <is>
           <t>90-110K€</t>
         </is>
       </c>
       <c r="P25" s="40" t="n"/>
-      <c r="Q25" s="42" t="inlineStr">
-        <is>
-          <t>18/06/2026</t>
-        </is>
-      </c>
+      <c r="Q25" s="42" t="n"/>
     </row>
     <row r="26" hidden="1" ht="40" customHeight="1">
       <c r="A26" s="77" t="inlineStr">
@@ -2652,17 +2652,17 @@
       <c r="C26" s="40" t="n"/>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Consultant Manager SIRH - HR Transformation</t>
+          <t>Responsable SIRH F/H</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Sopra Steria</t>
+          <t>KPMG France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>careers.soprasteria.com</t>
+          <t>Welcome to the Jungle / emplois.kpmg.fr</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Courbevoie (92)</t>
+          <t>Courbevoie / La Défense</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -2682,24 +2682,24 @@
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>Non affiché (2j télétravail/semaine)</t>
+          <t>Non affiché</t>
         </is>
       </c>
       <c r="K26" s="6" t="n"/>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>Sopra Steria, Consultant Manager = niveau senior (manage clients + junior consultants). HR Transformation paie + GTA + SIRH. Dossiers complexes, missions variées. 2j/sem télétravail. Big IT services France.</t>
+          <t>KPMG migration PeopleSoft → SAP SuccessFactors. Responsable SIRH = manager équipe + pilote roadmap. Requis 10 ans+ SIRH + team management + Core HR. Parfait fit Gaëtan (14 ans SAP + L'Oréal 40 pays). Démarrage mars 2026.</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>https://careers.soprasteria.com/job/consultant-manager-sirh-hr-transformation-ile-de-france-in-courbevoie-france-jid-792</t>
+          <t>https://www.welcometothejungle.com/fr/companies/kpmg-france/jobs/responsable-sirh-f-h_courbevoie</t>
         </is>
       </c>
       <c r="N26" s="40" t="n"/>
       <c r="O26" s="40" t="inlineStr">
         <is>
-          <t>70-85K€</t>
+          <t>90-110K€</t>
         </is>
       </c>
       <c r="P26" s="40" t="n"/>
@@ -2715,19 +2715,25 @@
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="C27" s="40" t="n"/>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Consultant SAP HCM (H/F)</t>
+          <t>Consultant Manager SIRH - HR Transformation</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>HR Path</t>
+          <t>Sopra Steria</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>jobs.hr-path.com</t>
+          <t>careers.soprasteria.com</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -2737,7 +2743,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq (59)</t>
+          <t>Courbevoie (92)</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -2745,28 +2751,29 @@
           <t>Partiel</t>
         </is>
       </c>
-      <c r="J27" s="6" t="n"/>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>Non affiché (2j télétravail/semaine)</t>
+        </is>
+      </c>
       <c r="K27" s="6" t="n"/>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>HR Path spécialiste SAP HCM/SF, posté 19/07/2026</t>
+          <t>Sopra Steria, Consultant Manager = niveau senior (manage clients + junior consultants). HR Transformation paie + GTA + SIRH. Dossiers complexes, missions variées. 2j/sem télétravail. Big IT services France.</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.hr-path.com/job/Villeneuve-d'Ascq-Consultant-SAP-HCM-(HF)-59-59650/770170201/</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>CV_GaetanFRANCOIS_CSM.html</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>650-750€/j</t>
-        </is>
-      </c>
+          <t>https://careers.soprasteria.com/job/consultant-manager-sirh-hr-transformation-ile-de-france-in-courbevoie-france-jid-792</t>
+        </is>
+      </c>
+      <c r="N27" s="40" t="n"/>
+      <c r="O27" s="40" t="inlineStr">
+        <is>
+          <t>70-85K€</t>
+        </is>
+      </c>
+      <c r="P27" s="40" t="n"/>
       <c r="Q27" s="42" t="inlineStr">
         <is>
           <t>18/06/2026</t>
@@ -2774,14 +2781,14 @@
       </c>
     </row>
     <row r="28" hidden="1" ht="40" customHeight="1">
-      <c r="A28" s="78" t="inlineStr">
+      <c r="A28" s="77" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Consultant SAP SuccessFactors (H/F)</t>
+          <t>Consultant SAP HCM (H/F)</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2801,7 +2808,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Paris La Défense</t>
+          <t>Villeneuve-d'Ascq (59)</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -2813,12 +2820,12 @@
       <c r="K28" s="6" t="n"/>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>HR Path leader SAP HCM/SF, posté 16/07/2026</t>
+          <t>HR Path spécialiste SAP HCM/SF, posté 19/07/2026</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.hr-path.com/job/Paris-La-D%C3%A9fense-Cedex-Consultant-SAP-SuccessFactors-(HF)-75-92042/818651901/</t>
+          <t>https://jobs.hr-path.com/job/Villeneuve-d'Ascq-Consultant-SAP-HCM-(HF)-59-59650/770170201/</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2831,7 +2838,11 @@
           <t>650-750€/j</t>
         </is>
       </c>
-      <c r="Q28" s="42" t="n"/>
+      <c r="Q28" s="42" t="inlineStr">
+        <is>
+          <t>18/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="29" hidden="1" ht="40" customHeight="1">
       <c r="A29" s="78" t="inlineStr">
@@ -2841,7 +2852,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Consultant SIRH (H/F) - Workday / Oracle HCM / SAP SuccessFactors</t>
+          <t>Consultant SAP SuccessFactors (H/F)</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -2873,12 +2884,12 @@
       <c r="K29" s="6" t="n"/>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>Multi-SIRH, posté 27/07/2026 - très récent</t>
+          <t>HR Path leader SAP HCM/SF, posté 16/07/2026</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.hr-path.com/job/Paris-La-D%C3%A9fense-Cedex-Consultant-SIRH-(HF)-Workday-%E2%80%A2-Oracle-HCM-%E2%80%A2-SAP-SuccessFactors-75-92042/1419350533/</t>
+          <t>https://jobs.hr-path.com/job/Paris-La-D%C3%A9fense-Cedex-Consultant-SAP-SuccessFactors-(HF)-75-92042/818651901/</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2888,14 +2899,10 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>650-750€/j ou 70-85K€</t>
-        </is>
-      </c>
-      <c r="Q29" s="42" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
+          <t>650-750€/j</t>
+        </is>
+      </c>
+      <c r="Q29" s="42" t="n"/>
     </row>
     <row r="30" hidden="1" ht="40" customHeight="1">
       <c r="A30" s="78" t="inlineStr">
@@ -2905,17 +2912,17 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Consultant SAP HCM Paie Senior</t>
+          <t>Consultant SIRH (H/F) - Workday / Oracle HCM / SAP SuccessFactors</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Strada (ex-Alight)</t>
+          <t>HR Path</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>careers.alight.com</t>
+          <t>jobs.hr-path.com</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2925,7 +2932,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Colombes, France</t>
+          <t>Paris La Défense</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -2937,12 +2944,12 @@
       <c r="K30" s="6" t="n"/>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>Strada = 1er partenaire SAP HR monde, 8000+ experts. Posté 2026. Parfait fit expertise L'Oréal/SAP HCM paie</t>
+          <t>Multi-SIRH, posté 27/07/2026 - très récent</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>https://careers.alight.com/strada/us/en/job/ALIGUSR27911STRADAENUS/Consultant-SAP-HCM-Paie-senior</t>
+          <t>https://jobs.hr-path.com/job/Paris-La-D%C3%A9fense-Cedex-Consultant-SIRH-(HF)-Workday-%E2%80%A2-Oracle-HCM-%E2%80%A2-SAP-SuccessFactors-75-92042/1419350533/</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2969,7 +2976,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Consultant SAP HCM Time Senior</t>
+          <t>Consultant SAP HCM Paie Senior</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -3001,12 +3008,12 @@
       <c r="K31" s="6" t="n"/>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>Strada expert SAP HCM Time, posté 2026</t>
+          <t>Strada = 1er partenaire SAP HR monde, 8000+ experts. Posté 2026. Parfait fit expertise L'Oréal/SAP HCM paie</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>https://careers.alight.com/strada/us/en/job/ALIGUSR27913STRADAENUS/Consultant-SAP-HCM-Time-senior</t>
+          <t>https://careers.alight.com/strada/us/en/job/ALIGUSR27911STRADAENUS/Consultant-SAP-HCM-Paie-senior</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3026,24 +3033,24 @@
       </c>
     </row>
     <row r="32" hidden="1" ht="16" customHeight="1">
-      <c r="A32" s="77" t="inlineStr">
+      <c r="A32" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Consultant SAP SuccessFactors expérimenté (H/F)</t>
+          <t>Consultant SAP HCM Time Senior</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>SQORUS</t>
+          <t>Strada (ex-Alight)</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn / fr.trabajo.org</t>
+          <t>careers.alight.com</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -3053,7 +3060,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Colombes, France</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -3061,20 +3068,16 @@
           <t>Partiel</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>60-75K€</t>
-        </is>
-      </c>
+      <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>SQORUS Great Place to Work 8 ans, 1500+ missions CAC40/SBF120. SAP SF expert, posté il y a 1 jour (28/07/2026). Très récent.</t>
+          <t>Strada expert SAP HCM Time, posté 2026</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>https://www.sqorus.com/carrieres/</t>
+          <t>https://careers.alight.com/strada/us/en/job/ALIGUSR27913STRADAENUS/Consultant-SAP-HCM-Time-senior</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3084,34 +3087,34 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>70-85K€</t>
+          <t>650-750€/j ou 70-85K€</t>
         </is>
       </c>
       <c r="Q32" s="42" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
     </row>
     <row r="33" hidden="1" ht="16" customHeight="1">
-      <c r="A33" s="78" t="inlineStr">
+      <c r="A33" s="77" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Principal Solution Advisor, HCM (F/H)</t>
+          <t>Consultant SAP SuccessFactors expérimenté (H/F)</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>SQORUS</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>LinkedIn / fr.trabajo.org</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -3121,57 +3124,65 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Levallois-Perret</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Hybride</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="n"/>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>60-75K€</t>
+        </is>
+      </c>
       <c r="K33" s="6" t="n"/>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>SAP pre-sales HCM, posté il y a 4 jours. Profil solution advisor senior, 14 ans SAP = fit parfait. Même famille que le poste SAP SuccessFactors déjà identifié.</t>
+          <t>SQORUS Great Place to Work 8 ans, 1500+ missions CAC40/SBF120. SAP SF expert, posté il y a 1 jour (28/07/2026). Très récent.</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.sap.com/go/SAP-Jobs-in-France/850401/</t>
+          <t>https://www.sqorus.com/carrieres/</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>CV_GaetanFRANCOIS_CSM_EN.html</t>
+          <t>CV_GaetanFRANCOIS_CSM.html</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>95-115K€</t>
-        </is>
-      </c>
-      <c r="Q33" s="42" t="n"/>
+          <t>70-85K€</t>
+        </is>
+      </c>
+      <c r="Q33" s="42" t="inlineStr">
+        <is>
+          <t>18/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="34" hidden="1" ht="48" customHeight="1">
-      <c r="A34" s="77" t="inlineStr">
+      <c r="A34" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Consultant(e) AMOA SIRH (F/H)</t>
+          <t>Principal Solution Advisor, HCM (F/H)</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>ACT-ON HRIS</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>SmartRecruiters / LinkedIn</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -3181,41 +3192,37 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Neuilly-sur-Seine</t>
+          <t>Levallois-Perret</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Hybride</t>
         </is>
       </c>
       <c r="J34" s="6" t="n"/>
       <c r="K34" s="6" t="n"/>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>ACT-ON HRIS 600+ consultants, 65M€ CA, 1 500+ missions. AMOA SIRH multi-outils (HR Access, Meta4, SAP SF). Posté juillet 2026. Postes actifs en juillet 2026, différent du poste AMOA déjà dans tableur.</t>
+          <t>SAP pre-sales HCM, posté il y a 4 jours. Profil solution advisor senior, 14 ans SAP = fit parfait. Même famille que le poste SAP SuccessFactors déjà identifié.</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/ACT-ON/744000045913473-consultant-e-amoa-sirh-f-h-</t>
+          <t>https://jobs.sap.com/go/SAP-Jobs-in-France/850401/</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>CV_GaetanFRANCOIS_CSM.html</t>
+          <t>CV_GaetanFRANCOIS_CSM_EN.html</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>70-85K€</t>
-        </is>
-      </c>
-      <c r="Q34" s="42" t="inlineStr">
-        <is>
-          <t>18/06/2026</t>
-        </is>
-      </c>
+          <t>95-115K€</t>
+        </is>
+      </c>
+      <c r="Q34" s="42" t="n"/>
     </row>
     <row r="35" hidden="1" ht="16" customHeight="1">
       <c r="A35" s="77" t="inlineStr">
@@ -3225,17 +3232,17 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Principal Solution Advisor, SuccessFactors (F/H)</t>
+          <t>Consultant(e) AMOA SIRH (F/H)</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>ACT-ON HRIS</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn / SAP Jobs France</t>
+          <t>SmartRecruiters / LinkedIn</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -3245,7 +3252,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Levallois-Perret (92)</t>
+          <t>Neuilly-sur-Seine</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -3257,22 +3264,22 @@
       <c r="K35" s="6" t="n"/>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>Poste pre-sales HCM senior SAP France, publié ~24/07/2026 (il y a 6 jours). 10-15 ans expérience SAP requis dont 3-5 ans HCM, Cloud SaaS B2B, anglais+français. Fit exceptionnel : 14 ans SAP HR, L'Oréal 40 pays, profil face client. Voir jobs.sap.com/go/SAP-Jobs-in-France/850401/ pour le lien actif.</t>
+          <t>ACT-ON HRIS 600+ consultants, 65M€ CA, 1 500+ missions. AMOA SIRH multi-outils (HR Access, Meta4, SAP SF). Posté juillet 2026. Postes actifs en juillet 2026, différent du poste AMOA déjà dans tableur.</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/principal-solution-advisor-successfactors-f-h-at-sap-4415727184</t>
+          <t>https://jobs.smartrecruiters.com/ACT-ON/744000045913473-consultant-e-amoa-sirh-f-h-</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>CV_GaetanFRANCOIS_CSM_EN.html</t>
+          <t>CV_GaetanFRANCOIS_CSM.html</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>95-115K€</t>
+          <t>70-85K€</t>
         </is>
       </c>
       <c r="Q35" s="42" t="inlineStr">
@@ -3282,24 +3289,24 @@
       </c>
     </row>
     <row r="36" hidden="1" ht="16" customHeight="1">
-      <c r="A36" s="78" t="inlineStr">
+      <c r="A36" s="77" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Consultant Senior HR Transformation - SAP SuccessFactors (F/H)</t>
+          <t>Principal Solution Advisor, SuccessFactors (F/H)</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Welcome to the Jungle</t>
+          <t>LinkedIn / SAP Jobs France</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -3309,37 +3316,41 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Levallois-Perret (92)</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>Hybride</t>
+          <t>Partiel</t>
         </is>
       </c>
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>Deloitte Human Capital. Pilotage projets SAP SuccessFactors, ateliers métier, déploiement opérationnel, certifications SF proposées. 5-10 ans SIRH requis. Fit excellent croisement SAP HR + conseil grands comptes.</t>
+          <t>Poste pre-sales HCM senior SAP France, publié ~24/07/2026 (il y a 6 jours). 10-15 ans expérience SAP requis dont 3-5 ans HCM, Cloud SaaS B2B, anglais+français. Fit exceptionnel : 14 ans SAP HR, L'Oréal 40 pays, profil face client. Voir jobs.sap.com/go/SAP-Jobs-in-France/850401/ pour le lien actif.</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/fr/companies/deloitte/jobs/consultant-senior-hr-transformation-sap-successfactors-f-h_paris</t>
+          <t>https://fr.linkedin.com/jobs/view/principal-solution-advisor-successfactors-f-h-at-sap-4415727184</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>CV_GaetanFRANCOIS_CSM.html</t>
+          <t>CV_GaetanFRANCOIS_CSM_EN.html</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>70-85K€</t>
-        </is>
-      </c>
-      <c r="Q36" s="42" t="n"/>
+          <t>95-115K€</t>
+        </is>
+      </c>
+      <c r="Q36" s="42" t="inlineStr">
+        <is>
+          <t>18/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="32" customHeight="1">
       <c r="A37" s="78" t="inlineStr">
@@ -3349,12 +3360,12 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Responsable SIRH F/H (migration PeopleSoft → SAP SuccessFactors)</t>
+          <t>Consultant Senior HR Transformation - SAP SuccessFactors (F/H)</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>KPMG France</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -3369,24 +3380,24 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>La Défense (92)</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Hybride</t>
         </is>
       </c>
       <c r="J37" s="6" t="n"/>
       <c r="K37" s="6" t="n"/>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>Poste interne KPMG : manager la migration PeopleSoft vers SAP SuccessFactors, management d'équipe. Min. 10 ans SIRH. Pas un poste conseil mais fit technique exceptionnel — migration SAP HR = coeur du profil. KPMG groupe international 180+ pays.</t>
+          <t>Deloitte Human Capital. Pilotage projets SAP SuccessFactors, ateliers métier, déploiement opérationnel, certifications SF proposées. 5-10 ans SIRH requis. Fit excellent croisement SAP HR + conseil grands comptes.</t>
         </is>
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/fr/companies/kpmg-france/jobs/responsable-sirh-f-h_courbevoie</t>
+          <t>https://www.welcometothejungle.com/fr/companies/deloitte/jobs/consultant-senior-hr-transformation-sap-successfactors-f-h_paris</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3396,14 +3407,10 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>90-110K€</t>
-        </is>
-      </c>
-      <c r="Q37" s="42" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
+          <t>70-85K€</t>
+        </is>
+      </c>
+      <c r="Q37" s="42" t="n"/>
     </row>
     <row r="38" hidden="1" ht="16" customHeight="1">
       <c r="A38" s="78" t="inlineStr">
@@ -3413,17 +3420,17 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Consultant SIRH Senior/Lead (Workday / Oracle HCM / SAP SuccessFactors) H/F</t>
+          <t>Responsable SIRH F/H (migration PeopleSoft → SAP SuccessFactors)</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>HR Path</t>
+          <t>KPMG France</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>jobs.hr-path.com</t>
+          <t>Welcome to the Jungle</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -3433,24 +3440,24 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>Paris La Défense</t>
+          <t>La Défense (92)</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>Hybride</t>
+          <t>Partiel</t>
         </is>
       </c>
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="6" t="n"/>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>Publié 27/07/2026. Niveau Senior/Lead/Chef de projet SIRH, projets internationaux, min. 4 ans SIRH, Workday ou Oracle HCM ou SAP SF, anglais professionnel. HR Path = spécialiste #1 RH tech Europe. Fit excellent — senior assumé dans l'intitulé.</t>
+          <t>Poste interne KPMG : manager la migration PeopleSoft vers SAP SuccessFactors, management d'équipe. Min. 10 ans SIRH. Pas un poste conseil mais fit technique exceptionnel — migration SAP HR = coeur du profil. KPMG groupe international 180+ pays.</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.hr-path.com/job/Paris-La-D%C3%A9fense-Cedex-Consultant-SIRH-%28HF%29-Workday-%E2%80%A2-Oracle-HCM-%E2%80%A2-SAP-SuccessFactors-75-92042/1419350533/</t>
+          <t>https://www.welcometothejungle.com/fr/companies/kpmg-france/jobs/responsable-sirh-f-h_courbevoie</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3460,7 +3467,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>70-85K€</t>
+          <t>90-110K€</t>
         </is>
       </c>
       <c r="Q38" s="42" t="inlineStr">
@@ -3477,17 +3484,17 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Consultant SAP HCM Paie senior</t>
+          <t>Consultant SIRH Senior/Lead (Workday / Oracle HCM / SAP SuccessFactors) H/F</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Strada (ex-Alight / ex-NGA Human Resources)</t>
+          <t>HR Path</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>careers.alight.com/strada</t>
+          <t>jobs.hr-path.com</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -3497,109 +3504,105 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Colombes (92)</t>
+          <t>Paris La Défense</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>Oui (depuis toute la France)</t>
+          <t>Hybride</t>
         </is>
       </c>
       <c r="J39" s="6" t="n"/>
       <c r="K39" s="6" t="n"/>
       <c r="L39" s="5" t="inlineStr">
         <is>
+          <t>Publié 27/07/2026. Niveau Senior/Lead/Chef de projet SIRH, projets internationaux, min. 4 ans SIRH, Workday ou Oracle HCM ou SAP SF, anglais professionnel. HR Path = spécialiste #1 RH tech Europe. Fit excellent — senior assumé dans l'intitulé.</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>https://jobs.hr-path.com/job/Paris-La-D%C3%A9fense-Cedex-Consultant-SIRH-%28HF%29-Workday-%E2%80%A2-Oracle-HCM-%E2%80%A2-SAP-SuccessFactors-75-92042/1419350533/</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>CV_GaetanFRANCOIS_CSM.html</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>70-85K€</t>
+        </is>
+      </c>
+      <c r="Q39" s="42" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="78" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Consultant SAP HCM Paie senior</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Strada (ex-Alight / ex-NGA Human Resources)</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>careers.alight.com/strada</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>Colombes (92)</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>Oui (depuis toute la France)</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="n"/>
+      <c r="K40" s="6" t="n"/>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
           <t>Strada = 1er partenaire mondial SAP HR. Configuration payroll SAP HCM France (cycles, schémas, contributions, accounting). 5+ ans SAP HCM Payroll requis. Fit parfait. Remote depuis toute la France confirmé. 2 annonces actives (R-27911 et R-32021).</t>
         </is>
       </c>
-      <c r="M39" s="5" t="inlineStr">
+      <c r="M40" s="5" t="inlineStr">
         <is>
           <t>https://careers.alight.com/strada/us/en/job/ALIGUSR32021STRADAENUS/Consultant-SAP-HCM-Paie-senior</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>CV_GaetanFRANCOIS_CSM.html</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>70-85K€</t>
         </is>
       </c>
-      <c r="Q39" s="42" t="inlineStr">
+      <c r="Q40" s="42" t="inlineStr">
         <is>
           <t>06/07/2026</t>
         </is>
       </c>
-    </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="77" t="inlineStr">
-        <is>
-          <t>⭐⭐⭐⭐⭐</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Consultant SAP Paie HCM Payroll</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Client via Duonext</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>free-work.com</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>Freelance</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>Département 92</t>
-        </is>
-      </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>Hybride (2-3j/semaine sur site)</t>
-        </is>
-      </c>
-      <c r="J40" s="6" t="inlineStr">
-        <is>
-          <t>650-750€/j</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="inlineStr">
-        <is>
-          <t>6 mois min. renouvelables</t>
-        </is>
-      </c>
-      <c r="L40" s="5" t="inlineStr">
-        <is>
-          <t>Publié 22/06/2026. Démarrage septembre 2026. Transformation RH, expertise paie France obligatoire (DSN, contributions, accounting), 8-10 ans requis. Très bon fit L'Oréal paie France multisite.</t>
-        </is>
-      </c>
-      <c r="M40" s="5" t="inlineStr">
-        <is>
-          <t>https://www.free-work.com/fr/tech-it/job-mission/consultant-erp-ms-dynamics-oracle-sage-sap/consultant-sap-paie-hcm-payroll</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>CV_GaetanFRANCOIS_CSM.html</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>650-750€/j</t>
-        </is>
-      </c>
-      <c r="Q40" s="42" t="n"/>
     </row>
     <row r="41" hidden="1" ht="16" customHeight="1">
       <c r="A41" s="77" t="inlineStr">
@@ -3609,217 +3612,221 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
+          <t>Consultant SAP Paie HCM Payroll</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Client via Duonext</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>free-work.com</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>Département 92</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>Hybride (2-3j/semaine sur site)</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>650-750€/j</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>6 mois min. renouvelables</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>Publié 22/06/2026. Démarrage septembre 2026. Transformation RH, expertise paie France obligatoire (DSN, contributions, accounting), 8-10 ans requis. Très bon fit L'Oréal paie France multisite.</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>https://www.free-work.com/fr/tech-it/job-mission/consultant-erp-ms-dynamics-oracle-sage-sap/consultant-sap-paie-hcm-payroll</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>CV_GaetanFRANCOIS_CSM.html</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>650-750€/j</t>
+        </is>
+      </c>
+      <c r="Q41" s="42" t="n"/>
+    </row>
+    <row r="42" hidden="1" ht="16" customHeight="1">
+      <c r="A42" s="77" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
           <t>SAP HCM Technico-Functional Consultant French Payroll</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>Apps IT Limited</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F42" s="5" t="inlineStr">
         <is>
           <t>free-work.com</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>Freelance</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
         <is>
           <t>Oui (100% remote)</t>
         </is>
       </c>
-      <c r="J41" s="6" t="inlineStr">
+      <c r="J42" s="6" t="inlineStr">
         <is>
           <t>650-750€/j</t>
         </is>
       </c>
-      <c r="K41" s="6" t="inlineStr">
+      <c r="K42" s="6" t="inlineStr">
         <is>
           <t>6 mois</t>
         </is>
       </c>
-      <c r="L41" s="5" t="inlineStr">
+      <c r="L42" s="5" t="inlineStr">
         <is>
           <t>Publié 17/06/2026. 100% remote — fit parfait pour Anglet. Profil technico-fonctionnel SAP HCM French Payroll. À vérifier disponibilité (publié il y a 6 semaines). Lien : rechercher "Apps IT" sur free-work.com/fr/tech-it/jobs/sap-hcm.</t>
         </is>
       </c>
-      <c r="M41" s="5" t="inlineStr">
+      <c r="M42" s="5" t="inlineStr">
         <is>
           <t>https://www.free-work.com/fr/tech-it/jobs/sap-hcm</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>CV_GaetanFRANCOIS_CSM.html</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t>650-750€/j</t>
         </is>
       </c>
-      <c r="Q41" s="42" t="n"/>
-    </row>
-    <row r="42" hidden="1" ht="16" customHeight="1">
-      <c r="A42" s="78" t="inlineStr">
+      <c r="Q42" s="42" t="n"/>
+    </row>
+    <row r="43" hidden="1" ht="16" customHeight="1">
+      <c r="A43" s="78" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>SAP HCM Consultant French Payroll</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>Client via Movement Group</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F43" s="5" t="inlineStr">
         <is>
           <t>movementgroup.uk</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>Freelance</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="I42" s="6" t="inlineStr">
+      <c r="I43" s="6" t="inlineStr">
         <is>
           <t>Oui (100% remote)</t>
         </is>
       </c>
-      <c r="J42" s="6" t="inlineStr">
+      <c r="J43" s="6" t="inlineStr">
         <is>
           <t>650-750€/j</t>
         </is>
       </c>
-      <c r="K42" s="6" t="inlineStr">
+      <c r="K43" s="6" t="inlineStr">
         <is>
           <t>12 mois + extension</t>
         </is>
       </c>
-      <c r="L42" s="5" t="inlineStr">
+      <c r="L43" s="5" t="inlineStr">
         <is>
           <t>Movement Group = cabinet recrutement SAP UK/Europe. 100% remote, 12 mois extensible. Outside IR35 (client probablement UK/international). 3+ ans SAP Payroll France requis. Durée et remote = fit parfait.</t>
         </is>
       </c>
-      <c r="M42" s="5" t="inlineStr">
+      <c r="M43" s="5" t="inlineStr">
         <is>
           <t>https://movementgroup.uk/job/sap-hcm-consultant-time-management/</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>CV_GaetanFRANCOIS_CSM_EN.html</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>650-750€/j</t>
         </is>
       </c>
-      <c r="Q42" s="42" t="n"/>
-    </row>
-    <row r="43" hidden="1" ht="16" customHeight="1">
-      <c r="A43" s="77" t="inlineStr">
+      <c r="Q43" s="42" t="n"/>
+    </row>
+    <row r="44" hidden="1" ht="32" customHeight="1">
+      <c r="A44" s="77" t="inlineStr">
         <is>
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Consultant(e) AMOA SIRH (F/H)</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>ACT-ON HRIS</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>SmartRecruiters / LinkedIn</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>Neuilly-sur-Seine (92)</t>
-        </is>
-      </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>Partiel</t>
-        </is>
-      </c>
-      <c r="J43" s="6" t="n"/>
-      <c r="K43" s="6" t="n"/>
-      <c r="L43" s="5" t="inlineStr">
-        <is>
-          <t>ACT-ON HRIS filiale SIRH du groupe ACT-ON (600+ collab., 65M€ CA). Profil exact : SAP SuccessFactors, HR Access, AMOA, specs fonctionnelles, conduite du changement. 15 ans SAP + 40 pays L'Oréal = profil senior idéal. Lien : jobs.smartrecruiters.com/ACT-ON/744000045913473</t>
-        </is>
-      </c>
-      <c r="M43" s="5" t="inlineStr">
-        <is>
-          <t>https://jobs.smartrecruiters.com/ACT-ON/744000045913473-consultant-e-amoa-sirh-f-h-</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>CV_GaetanFRANCOIS_CSM.html</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>75-85K€</t>
-        </is>
-      </c>
-      <c r="Q43" s="42" t="inlineStr">
-        <is>
-          <t>18/06/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" hidden="1" ht="32" customHeight="1">
-      <c r="A44" s="78" t="inlineStr">
-        <is>
-          <t>⭐⭐⭐⭐⭐</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Consultant(e) SuccessFactors (F/H)</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>ACT-ON HRIS</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -3841,12 +3848,12 @@
       <c r="K44" s="6" t="n"/>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>Poste SAP SuccessFactors dédié chez ACT-ON HRIS, publié il y a 2 jours — fenêtre idéale pour postuler. Gaëtan cumule 14 ans SAP HR/HCM ; correspond exactement au profil recherché par ce cabinet spécialisé HumanTech.</t>
+          <t>ACT-ON HRIS filiale SIRH du groupe ACT-ON (600+ collab., 65M€ CA). Profil exact : SAP SuccessFactors, HR Access, AMOA, specs fonctionnelles, conduite du changement. 15 ans SAP + 40 pays L'Oréal = profil senior idéal. Lien : jobs.smartrecruiters.com/ACT-ON/744000045913473</t>
         </is>
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/consultant-e-successfactors-f-h-at-act-on-hris</t>
+          <t>https://jobs.smartrecruiters.com/ACT-ON/744000045913473-consultant-e-amoa-sirh-f-h-</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3859,7 +3866,11 @@
           <t>75-85K€</t>
         </is>
       </c>
-      <c r="Q44" s="42" t="n"/>
+      <c r="Q44" s="42" t="inlineStr">
+        <is>
+          <t>18/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="45" hidden="1" ht="32" customHeight="1">
       <c r="A45" s="78" t="inlineStr">
@@ -3869,7 +3880,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Consultant Confirmé SIRH - SAP HR (H/F)</t>
+          <t>Consultant(e) SuccessFactors (F/H)</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3901,12 +3912,12 @@
       <c r="K45" s="6" t="n"/>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>Poste SAP HR publié ce matin même (31/07/2026, il y a 17h) — postuler en priorité absolue aujourd'hui. Intitulé "Confirmé" = niveau intermédiaire, Gaëtan au-dessus, peut négocier un niveau senior. ACT-ON HRIS = cabinet SIRH pur spécialisé.</t>
+          <t>Poste SAP SuccessFactors dédié chez ACT-ON HRIS, publié il y a 2 jours — fenêtre idéale pour postuler. Gaëtan cumule 14 ans SAP HR/HCM ; correspond exactement au profil recherché par ce cabinet spécialisé HumanTech.</t>
         </is>
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/consultant-confirme-sirh-sap-hr-h-f-at-act-on-hris</t>
+          <t>https://fr.linkedin.com/jobs/view/consultant-e-successfactors-f-h-at-act-on-hris</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3919,11 +3930,7 @@
           <t>75-85K€</t>
         </is>
       </c>
-      <c r="Q45" s="42" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
+      <c r="Q45" s="42" t="n"/>
     </row>
     <row r="46" ht="32" customHeight="1">
       <c r="A46" s="78" t="inlineStr">
@@ -3931,25 +3938,19 @@
           <t>⭐⭐⭐⭐⭐</t>
         </is>
       </c>
-      <c r="B46" s="40" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="C46" s="40" t="n"/>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>HRIS &amp; AI Tech Pre-Sales Specialist</t>
+          <t>Consultant Confirmé SIRH - SAP HR (H/F)</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Arago Consulting</t>
+          <t>ACT-ON HRIS</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>SmartRecruiters</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -3959,37 +3960,36 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>Paris ou Bordeaux</t>
+          <t>Neuilly-sur-Seine (92)</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>Partiel (déplacements clients)</t>
+          <t>Partiel</t>
         </is>
       </c>
       <c r="J46" s="6" t="n"/>
       <c r="K46" s="6" t="n"/>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>Arago = 1er partenaire européen SAP SuccessFactors. Croisement parfait pre-sales IA+SIRH : 14 ans SAP, 40 pays L'Oréal, usage quotidien IA générative, profil face-client senior. Bordeaux = 2h d'Anglet. Lien : jobs.smartrecruiters.com/Arago/744000139094386</t>
+          <t>Poste SAP HR publié ce matin même (31/07/2026, il y a 17h) — postuler en priorité absolue aujourd'hui. Intitulé "Confirmé" = niveau intermédiaire, Gaëtan au-dessus, peut négocier un niveau senior. ACT-ON HRIS = cabinet SIRH pur spécialisé.</t>
         </is>
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/Arago/744000139094386-hris-ai-tech-pre-sales-specialist</t>
-        </is>
-      </c>
-      <c r="N46" s="40" t="inlineStr">
-        <is>
-          <t>Resume_GaetanFRANCOIS_Arago.pdf</t>
-        </is>
-      </c>
-      <c r="O46" s="40" t="inlineStr">
-        <is>
-          <t>90-110K€</t>
-        </is>
-      </c>
-      <c r="P46" s="40" t="n"/>
+          <t>https://fr.linkedin.com/jobs/view/consultant-confirme-sirh-sap-hr-h-f-at-act-on-hris</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>CV_GaetanFRANCOIS_CSM.html</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>75-85K€</t>
+        </is>
+      </c>
       <c r="Q46" s="42" t="inlineStr">
         <is>
           <t>06/07/2026</t>

</xml_diff>

<commit_message>
tableur: Qurated Global Product Owner SuccessFactors - postule 07/08/2026
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -28425,8 +28425,7 @@
     </filterColumn>
   </autoFilter>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -52471,7 +52470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q73"/>
+  <dimension ref="A1:Q74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="16" max="17"/>
@@ -57676,6 +57675,84 @@
       <c r="Q73" s="41" t="inlineStr">
         <is>
           <t>06/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="128" customHeight="1">
+      <c r="A74" s="67" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Postulé</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Global Product Owner - SuccessFactors</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Qurated (pour un cabinet d avocats international)</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>CDD / FTC 18 mois</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>100% remote</t>
+        </is>
+      </c>
+      <c r="J74" s="6" t="n"/>
+      <c r="K74" s="6" t="inlineStr">
+        <is>
+          <t>18 mois</t>
+        </is>
+      </c>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>Ownership unique de la plateforme SAP SuccessFactors sur tout le perimetre mondial : vision et roadmap, solution design multi-modules (Employee Central, Performance &amp; Goals, Compensation, Recruiting, Onboarding, Learning), standards globaux, cycles de release, conduite du changement et relation editeur. Fit tres eleve : SuccessFactors multi-modules, contexte global et conduite du changement correspondent au parcours L'Oreal. Full remote. Postule le 07/08/2026.</t>
+        </is>
+      </c>
+      <c r="M74" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4447393087</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_SIRH_EN.pdf</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rôle WallOfTraders.com en Product Manager partout + nouvel onglet Offres PM
Rôle : "Co-founder & Product Manager" (FR : "Co-fondateur & Product Manager")
dans les 20 CV concernés, en remplacement de CEO, Directeur Général, DG et
Associé. PDF régénérés, tous sur une page. Règle inscrite dans CLAUDE.md.

Correction de méthode : les CV_*.html sont en réalité au format sidebar comme
les Resume_*.html et doivent être générés avec "@page margin: 0". La marge
1.5cm/1.8cm documentée dans CLAUDE.md les faisait passer de 1 à 3 pages.

Nouvel onglet "Offres PM" avec routage automatique dans add_offre.py. Une offre
produit portant un marqueur SIRH ou SAP reste dans Offres SIRH. La détection IA
attrape désormais "IA" et "AI" comme mots isolés ("Expert IA", "Solutions IA"),
ce qui évite le tri manuel constaté le 13/08.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -9,13 +9,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offres SIRH" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offres CSM" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offres IA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fait" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Légende" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offres PM" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fait" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Légende" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Offres SIRH'!$A$1:$O$463</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Offres CSM'!$A$1:$O$295</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Offres IA'!$A$1:$O$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Offres PM'!$A$1:$O$1</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -98,7 +100,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="53">
+  <fills count="54">
     <fill>
       <patternFill/>
     </fill>
@@ -365,6 +367,11 @@
         <fgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD700"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -394,7 +401,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -609,6 +616,8 @@
     <xf numFmtId="0" fontId="7" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="53" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -35281,7 +35290,7 @@
       <c r="K48" s="6" t="n"/>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>Encadrement de l'équipe CSM EMEA chez un éditeur search/discovery ecommerce. Points forts : enterprise multi-pays, rôle d'escalade et interface Produit/Engineering (equivalent du role L1/L2/L3 chez L'Oreal), multilinguisme valorisé en bonus, full remote depuis la France. Sephora est client de Constructor : angle beaute/retail a exploiter en LM via L'Oreal et le deploiement Tamigo en magasins. ECART A ASSUMER : ils demandent d'avoir deja manage une equipe de CSM/TAM/Solutions Consulting ; le CV documente du management d'equipe offshore (Inde, 2014-2016), un alternant et le role de CEO cofondateur, pas du line management de CSM. Domaine search/ecommerce inconnu. Remplace l'ancienne annonce Constructor CSM French Speaker, fermee.</t>
+          <t>Encadrement de l'équipe CSM EMEA chez un éditeur search/discovery ecommerce. Points forts : enterprise multi-pays, rôle d'escalade et interface Produit/Engineering (equivalent du role L1/L2/L3 chez L'Oreal), multilinguisme valorisé en bonus, full remote depuis la France. Sephora est client de Constructor : angle beaute/retail a exploiter en LM via L'Oreal et le deploiement Tamigo en magasins. ECART A ASSUMER : ils demandent d'avoir deja manage une equipe de CSM/TAM/Solutions Consulting ; le CV documente du management d'equipe offshore (Inde, 2014-2016), un alternant et le role de cofondateur et Product Manager, pas du line management de CSM. Domaine search/ecommerce inconnu. Remplace l'ancienne annonce Constructor CSM French Speaker, fermee.</t>
         </is>
       </c>
       <c r="M48" s="5" t="inlineStr">
@@ -60392,6 +60401,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.6640625" customWidth="1" min="1" max="1"/>
+    <col width="10.83203125" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="51.83203125" customWidth="1" min="4" max="4"/>
+    <col width="25.5" customWidth="1" min="5" max="5"/>
+    <col width="21.5" customWidth="1" min="6" max="6"/>
+    <col width="14.1640625" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="23.6640625" customWidth="1" min="9" max="9"/>
+    <col width="26.6640625" customWidth="1" min="10" max="10"/>
+    <col width="17.33203125" customWidth="1" min="11" max="11"/>
+    <col width="99.83203125" customWidth="1" min="12" max="12"/>
+    <col width="106.5" customWidth="1" min="13" max="13"/>
+    <col width="31.33203125" customWidth="1" min="14" max="14"/>
+    <col width="9.1640625" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Fait</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>Entreprise</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>Contrat</t>
+        </is>
+      </c>
+      <c r="H1" s="14" t="inlineStr">
+        <is>
+          <t>Localisation</t>
+        </is>
+      </c>
+      <c r="I1" s="14" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="J1" s="14" t="inlineStr">
+        <is>
+          <t>Salaire / TJM</t>
+        </is>
+      </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>Durée mission</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="inlineStr">
+        <is>
+          <t>Fit / Notes</t>
+        </is>
+      </c>
+      <c r="M1" s="14" t="inlineStr">
+        <is>
+          <t>Lien</t>
+        </is>
+      </c>
+      <c r="N1" s="102" t="inlineStr">
+        <is>
+          <t>CV à envoyer</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Prétention</t>
+        </is>
+      </c>
+      <c r="P1" s="40" t="inlineStr">
+        <is>
+          <t>Date trouvée</t>
+        </is>
+      </c>
+      <c r="Q1" s="40" t="inlineStr">
+        <is>
+          <t>Date publiée</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Product Manager: Customer Onboarding Experience</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Constructor</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>jobs.ashbyhq.com</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Propriete du parcours d'integration client (SDK, docs, instrumentation de tracking), north star time-to-value. Atouts : propriete produit reelle chez WallOfTraders.com, parcours d'integration L'Oreal sur 40 pays, role de charniere metier/developpeurs, redaction de specifications. LACUNE DURE : ils exigent 3+ ans de PM sur produit oriente developpeurs (SDK, API, tracking) ; Gaetan n'en a pas, c'est un filtre potentiellement eliminatoire. Candidature plus risquee que le poste Regional Manager CS chez le meme employeur.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/constructor/e8fa6194-ef2e-47d3-ab45-a9112d87da24</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>80-100 K€</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Q107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
@@ -68203,7 +68394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
tableur: premiere recherche Product Manager - 18 offres dans Offres PM
Sources validées par API quand c'était possible (Ashby et Lever). Les postes
Deel, Dash0, EverAI, SignalWire et Workwize remontés par WebSearch étaient déjà
fermés et ont été écartés ; l'API le confirme là où le moteur de recherche
affichait encore les annonces.

Documente l'API publique Lever dans CLAUDE.md, avec l'avertissement Jobgether
(même offre dupliquée par pays, filtrer sur la variante France).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -100,7 +100,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="54">
+  <fills count="56">
     <fill>
       <patternFill/>
     </fill>
@@ -372,6 +372,16 @@
         <fgColor rgb="00FFD700"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF8C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -401,7 +411,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -618,6 +628,8 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="53" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="54" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="55" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -60401,7 +60413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.6640625" customWidth="1" min="1" max="1"/>
@@ -60510,64 +60522,1220 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="103" t="inlineStr">
+      <c r="A2" s="104" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Senior Product Manager - Core Platform (Remote)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Camunda</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>jobs.ashbyhq.com</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Editeur d'orchestration de processus, entreprise remote-first. Gaetan avait deja cible Camunda (CV_GaetanFRANCOIS_Camunda_EN existe), donc le contexte est connu. Poste verifie ouvert par l'API Ashby le 14/08.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/camunda/b771e145-a5cf-4867-ad13-b54830e3b744</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>85-100 K€</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="104" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Senior Product Builder - Connectors Experience - EMEA</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Camunda</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>jobs.ashbyhq.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Produit centre sur l'experience des connecteurs, donc sur l'integration : c'est l'angle le plus proche du parcours (parcours d'integration L'Oreal, charniere metier/developpeurs). Verifie ouvert par API.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/camunda/05cb2825-dcd9-40e6-bf92-bda409d99374</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>85-100 K€</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="104" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>360Learning</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>welcometothejungle.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Télétravail total</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Plateforme de learning : le domaine recoupe directement l'experience de formation utilisateurs-cles et de transfert de connaissances. Teletravail total, editeur francais bien etabli. Un des meilleurs croisements produit/parcours du lot.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://www.welcometothejungle.com/en/companies/360learning/jobs/product-manager_paris_360LE_lGeWWq1</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="104" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>welcometothejungle.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Télétravail total</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>55-59 K€</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Teletravail total, plus de 4 ans d'experience demandes, demarrage 31/08/2026. Remuneration sous la cible ; le salaire ne sert pas de filtre.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://www.welcometothejungle.com/fr/companies/side/jobs/product-manager_paris_SIDE_jRLO2Ar</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="104" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Inqom</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>welcometothejungle.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Paris / Tours</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Télétravail total</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>50-55 K€</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Teletravail total sur un SaaS comptable. Fourchette sous la cible, a negocier.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://www.welcometothejungle.com/fr/companies/inqom/jobs/product-manager</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="103" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Product Manager: Customer Onboarding Experience</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Constructor</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>jobs.ashbyhq.com</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Full remote</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Propriete du parcours d'integration client (SDK, docs, instrumentation de tracking), north star time-to-value. Atouts : propriete produit reelle chez WallOfTraders.com, parcours d'integration L'Oreal sur 40 pays, role de charniere metier/developpeurs, redaction de specifications. LACUNE DURE : ils exigent 3+ ans de PM sur produit oriente developpeurs (SDK, API, tracking) ; Gaetan n'en a pas, c'est un filtre potentiellement eliminatoire. Candidature plus risquee que le poste Regional Manager CS chez le meme employeur.</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/constructor/e8fa6194-ef2e-47d3-ab45-a9112d87da24</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>80-100 K€</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Product Manager, Self Managed Service</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Camunda</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>jobs.ashbyhq.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Troisieme poste produit ouvert chez Camunda ; perimetre self-managed, plus technique. Verifie ouvert par API.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/camunda/5652a3f3-e418-4e91-b58b-4be13f36853b</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>80-95 K€</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Product Manager (senior level)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Joko</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>welcometothejungle.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Télétravail total</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Niveau senior explicite, teletravail total. Produit B2C, ce qui recoupe l'experience WallOfTraders.com.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://www.welcometothejungle.com/en/companies/joko/jobs/product-manager-senior-level</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Product Manager (full remote avec déplacements)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>RISE</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>welcometothejungle.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Télétravail total</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Full remote avec deplacements ponctuels, compatible avec une base a Anglet.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://www.welcometothejungle.com/fr/companies/rise/jobs/28b1f52c-1924-40ec-b7e0-18bbdcda6c56</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Follow</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>welcometothejungle.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Télétravail total</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Teletravail total, secteur sante. A qualifier sur la seniorite attendue.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://www.welcometothejungle.com/fr/companies/follow-health/jobs/product-manager</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Product Manager, Data Activation</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>n.c. (via Jobgether)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>jobs.lever.co</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Remote depuis la France, verifie ouvert par l'API Lever. Jobgether publie la meme offre par pays ; seule la variante France est retenue ici.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/jobgether/dad5d8dc-4e02-4536-b7f6-8680e1df16ce</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Product Manager, Data Orchestration</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>n.c. (via Jobgether)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>jobs.lever.co</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Remote depuis la France, verifie ouvert par l'API Lever.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/jobgether/5245a149-8431-4452-ab44-50cbb9bafbcf</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>n.c. (via Jobgether)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>jobs.lever.co</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Product Owner en full remote depuis la France, verifie ouvert par l'API Lever.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/jobgether/5405e9ec-8ab3-4075-8f5e-96425e4f11a6</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>B2C Growth Product Manager</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>n.c. (via Jobgether)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>jobs.lever.co</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Produit B2C oriente growth : recoupe directement WallOfTraders.com (acquisition SEO, paid social, boucle de retour utilisateurs).</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/jobgether/bae287fc-687d-48a6-a860-100430cbe25e</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>75-90 K€</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Sr. Product Manager, Core Platform</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>n.c. (via Jobgether)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>jobs.lever.co</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>France / Pays-Bas</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Full remote</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Poste senior sur plateforme coeur, full remote.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/jobgether/3efb5da5-0c07-4209-a4b6-037ead7571c2</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>80-95 K€</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="103" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Senior Product Manager</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Pennylane</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>jobs.lever.co</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Remote Europe</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Scale-up francaise, remote depuis n'importe ou en Europe. URL issue de WebSearch : l'API Lever n'a pas repondu sur ce slug, verifier que l'annonce est encore ouverte avant de candidater.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/pennylane/e821e150-f513-4297-86a7-6d2ee25ac50c</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>80-95 K€</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="105" t="inlineStr">
+        <is>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ITSM Platform Architect / Technical Product Owner</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LeHibou</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>free-work</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Mission freelance</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>650 €/j</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>6 mois</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Product Owner technique sur plateforme ITSM. Sur site Paris, donc en retrait sur le critere remote.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>https://www.free-work.com/fr/tech-it/job-mission/product-owner/itsm-platform-architect-technical-product-owner</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>650 €/j</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="105" t="inlineStr">
+        <is>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Product Owner (H/F) 69</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Mindquest</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>free-work</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Mission freelance</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>400-550 €/j</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>3 mois</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Mission PO courte a Lyon, sur site.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>https://www.free-work.com/fr/tech-it/job-mission/product-owner/product-owner-h-f-69-1</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>550 €/j</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="105" t="inlineStr">
+        <is>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>WIKEYS</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>free-work</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Mission freelance</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Bruxelles</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>600-610 €/j</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>6 mois</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Mission PO a Bruxelles ; contexte international, mais sur site.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>https://www.free-work.com/fr/tech-it/job-mission/product-owner/product-owner-1365</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_Constructor_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>610 €/j</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CV produit: repositionnement product-first sur PM_EN/PM_FR et nouvelle variante plateforme B2B
- Sous-titre et profil des deux CV PM ouvrent desormais sur le role Product Manager
  chez WallOfTraders.com plutot que sur l'integration SaaS enterprise
- Nouveau Resume_GaetanFRANCOIS_PM_Platform_EN pour les 7 offres plateforme B2B
  de l'onglet Offres PM (Camunda x3, Constructor, Jobgether Core Platform,
  Data Activation, Data Orchestration)
- Colonne CV a envoyer mise a jour sur ces 7 lignes

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -15114,7 +15114,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -15176,7 +15176,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -15434,7 +15434,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -15496,7 +15496,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -15744,7 +15744,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -15806,7 +15806,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -15992,7 +15992,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">

</xml_diff>

<commit_message>
Offres PM: une seule candidature Camunda (Self Managed Service), les deux autres passees hors profil
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -15074,17 +15074,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Senior Product Manager - Core Platform (Remote)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Camunda</t>
+          <t>360Learning</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>jobs.ashbyhq.com</t>
+          <t>welcometothejungle.com</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -15094,32 +15094,32 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Full remote</t>
+          <t>Télétravail total</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Editeur d'orchestration de processus, entreprise remote-first. Gaetan avait deja cible Camunda (CV_GaetanFRANCOIS_Camunda_EN existe), donc le contexte est connu. Poste verifie ouvert par l'API Ashby le 14/08.</t>
+          <t>Plateforme de learning : le domaine recoupe directement l'experience de formation utilisateurs-cles et de transfert de connaissances. Teletravail total, editeur francais bien etabli. Un des meilleurs croisements produit/parcours du lot.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/camunda/b771e145-a5cf-4867-ad13-b54830e3b744</t>
+          <t>https://www.welcometothejungle.com/en/companies/360learning/jobs/product-manager_paris_360LE_lGeWWq1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_FR.pdf</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>85-100 K€</t>
+          <t>75-90 K€</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -15136,17 +15136,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Senior Product Builder - Connectors Experience - EMEA</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Camunda</t>
+          <t>Side</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>jobs.ashbyhq.com</t>
+          <t>welcometothejungle.com</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -15156,32 +15156,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Full remote</t>
+          <t>Télétravail total</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>55-59 K€</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Produit centre sur l'experience des connecteurs, donc sur l'integration : c'est l'angle le plus proche du parcours (parcours d'integration L'Oreal, charniere metier/developpeurs). Verifie ouvert par API.</t>
+          <t>Teletravail total, plus de 4 ans d'experience demandes, demarrage 31/08/2026. Remuneration sous la cible ; le salaire ne sert pas de filtre.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/camunda/05cb2825-dcd9-40e6-bf92-bda409d99374</t>
+          <t>https://www.welcometothejungle.com/fr/companies/side/jobs/product-manager_paris_SIDE_jRLO2Ar</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_FR.pdf</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>85-100 K€</t>
+          <t>75-90 K€</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -15203,7 +15208,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>360Learning</t>
+          <t>Inqom</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -15218,7 +15223,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Paris / Tours</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -15226,14 +15231,19 @@
           <t>Télétravail total</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>50-55 K€</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Plateforme de learning : le domaine recoupe directement l'experience de formation utilisateurs-cles et de transfert de connaissances. Teletravail total, editeur francais bien etabli. Un des meilleurs croisements produit/parcours du lot.</t>
+          <t>Teletravail total sur un SaaS comptable. Fourchette sous la cible, a negocier.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/en/companies/360learning/jobs/product-manager_paris_360LE_lGeWWq1</t>
+          <t>https://www.welcometothejungle.com/fr/companies/inqom/jobs/product-manager</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -15258,19 +15268,24 @@
           <t>⭐⭐⭐⭐</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Self Managed Service</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Side</t>
+          <t>Camunda</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>welcometothejungle.com</t>
+          <t>jobs.ashbyhq.com</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -15280,37 +15295,32 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Télétravail total</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>55-59 K€</t>
+          <t>Full remote</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Teletravail total, plus de 4 ans d'experience demandes, demarrage 31/08/2026. Remuneration sous la cible ; le salaire ne sert pas de filtre.</t>
+          <t>Seule candidature Camunda retenue. Le poste porte sur l'installation, la configuration et l'exploitation de Camunda 8 chez le client (on-premises, configurations enterprise, reduction de la friction de deploiement, travail avec pre-sales et solution architects) ; c'est le parcours SAP HR on-prem vers SuccessFactors. Lacune a concéder en LM : Kubernetes et Helm.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/fr/companies/side/jobs/product-manager_paris_SIDE_jRLO2Ar</t>
+          <t>https://jobs.ashbyhq.com/camunda/5652a3f3-e418-4e91-b58b-4be13f36853b</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_FR.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>75-90 K€</t>
+          <t>80-95 K€</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -15320,24 +15330,24 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="91" t="inlineStr">
-        <is>
-          <t>⭐⭐⭐⭐</t>
+      <c r="A6" s="90" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager: Customer Onboarding Experience</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Inqom</t>
+          <t>Constructor</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>welcometothejungle.com</t>
+          <t>jobs.ashbyhq.com</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -15347,37 +15357,32 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Paris / Tours</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Télétravail total</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>50-55 K€</t>
+          <t>Full remote</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Teletravail total sur un SaaS comptable. Fourchette sous la cible, a negocier.</t>
+          <t>Propriete du parcours d'integration client (SDK, docs, instrumentation de tracking), north star time-to-value. Atouts : propriete produit reelle chez WallOfTraders.com, parcours d'integration L'Oreal sur 40 pays, role de charniere metier/developpeurs, redaction de specifications. LACUNE DURE : ils exigent 3+ ans de PM sur produit oriente developpeurs (SDK, API, tracking) ; Gaetan n'en a pas, c'est un filtre potentiellement eliminatoire. Candidature plus risquee que le poste Regional Manager CS chez le meme employeur.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/fr/companies/inqom/jobs/product-manager</t>
+          <t>https://jobs.ashbyhq.com/constructor/e8fa6194-ef2e-47d3-ab45-a9112d87da24</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_FR.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>75-90 K€</t>
+          <t>80-100 K€</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -15394,17 +15399,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Product Manager: Customer Onboarding Experience</t>
+          <t>Product Manager (senior level)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Constructor</t>
+          <t>Joko</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>jobs.ashbyhq.com</t>
+          <t>welcometothejungle.com</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -15414,32 +15419,32 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Full remote</t>
+          <t>Télétravail total</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Propriete du parcours d'integration client (SDK, docs, instrumentation de tracking), north star time-to-value. Atouts : propriete produit reelle chez WallOfTraders.com, parcours d'integration L'Oreal sur 40 pays, role de charniere metier/developpeurs, redaction de specifications. LACUNE DURE : ils exigent 3+ ans de PM sur produit oriente developpeurs (SDK, API, tracking) ; Gaetan n'en a pas, c'est un filtre potentiellement eliminatoire. Candidature plus risquee que le poste Regional Manager CS chez le meme employeur.</t>
+          <t>Niveau senior explicite, teletravail total. Produit B2C, ce qui recoupe l'experience WallOfTraders.com.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/constructor/e8fa6194-ef2e-47d3-ab45-a9112d87da24</t>
+          <t>https://www.welcometothejungle.com/en/companies/joko/jobs/product-manager-senior-level</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>80-100 K€</t>
+          <t>75-90 K€</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -15456,17 +15461,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Product Manager, Self Managed Service</t>
+          <t>Product Manager (full remote avec déplacements)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Camunda</t>
+          <t>RISE</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>jobs.ashbyhq.com</t>
+          <t>welcometothejungle.com</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -15476,32 +15481,32 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>France</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Full remote</t>
+          <t>Télétravail total</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Troisieme poste produit ouvert chez Camunda ; perimetre self-managed, plus technique. Verifie ouvert par API.</t>
+          <t>Full remote avec deplacements ponctuels, compatible avec une base a Anglet.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/camunda/5652a3f3-e418-4e91-b58b-4be13f36853b</t>
+          <t>https://www.welcometothejungle.com/fr/companies/rise/jobs/28b1f52c-1924-40ec-b7e0-18bbdcda6c56</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_FR.pdf</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>80-95 K€</t>
+          <t>75-90 K€</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -15518,12 +15523,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Product Manager (senior level)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Joko</t>
+          <t>Follow</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -15538,7 +15543,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>France</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -15548,17 +15553,17 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Niveau senior explicite, teletravail total. Produit B2C, ce qui recoupe l'experience WallOfTraders.com.</t>
+          <t>Teletravail total, secteur sante. A qualifier sur la seniorite attendue.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/en/companies/joko/jobs/product-manager-senior-level</t>
+          <t>https://www.welcometothejungle.com/fr/companies/follow-health/jobs/product-manager</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_FR.pdf</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -15580,17 +15585,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Product Manager (full remote avec déplacements)</t>
+          <t>Product Manager, Data Activation</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>RISE</t>
+          <t>n.c. (via Jobgether)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>welcometothejungle.com</t>
+          <t>jobs.lever.co</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -15605,22 +15610,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Télétravail total</t>
+          <t>Full remote</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Full remote avec deplacements ponctuels, compatible avec une base a Anglet.</t>
+          <t>Remote depuis la France, verifie ouvert par l'API Lever. Jobgether publie la meme offre par pays ; seule la variante France est retenue ici.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/fr/companies/rise/jobs/28b1f52c-1924-40ec-b7e0-18bbdcda6c56</t>
+          <t>https://jobs.lever.co/jobgether/dad5d8dc-4e02-4536-b7f6-8680e1df16ce</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_FR.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -15642,17 +15647,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Data Orchestration</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Follow</t>
+          <t>n.c. (via Jobgether)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>welcometothejungle.com</t>
+          <t>jobs.lever.co</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -15667,22 +15672,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Télétravail total</t>
+          <t>Full remote</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Teletravail total, secteur sante. A qualifier sur la seniorite attendue.</t>
+          <t>Remote depuis la France, verifie ouvert par l'API Lever.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://www.welcometothejungle.com/fr/companies/follow-health/jobs/product-manager</t>
+          <t>https://jobs.lever.co/jobgether/5245a149-8431-4452-ab44-50cbb9bafbcf</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_FR.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -15704,7 +15709,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Product Manager, Data Activation</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -15734,17 +15739,17 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Remote depuis la France, verifie ouvert par l'API Lever. Jobgether publie la meme offre par pays ; seule la variante France est retenue ici.</t>
+          <t>Product Owner en full remote depuis la France, verifie ouvert par l'API Lever.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/jobgether/dad5d8dc-4e02-4536-b7f6-8680e1df16ce</t>
+          <t>https://jobs.lever.co/jobgether/5405e9ec-8ab3-4075-8f5e-96425e4f11a6</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -15766,7 +15771,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Product Manager, Data Orchestration</t>
+          <t>B2C Growth Product Manager</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -15796,17 +15801,17 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Remote depuis la France, verifie ouvert par l'API Lever.</t>
+          <t>Produit B2C oriente growth : recoupe directement WallOfTraders.com (acquisition SEO, paid social, boucle de retour utilisateurs).</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/jobgether/5245a149-8431-4452-ab44-50cbb9bafbcf</t>
+          <t>https://jobs.lever.co/jobgether/bae287fc-687d-48a6-a860-100430cbe25e</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -15828,7 +15833,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Sr. Product Manager, Core Platform</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -15848,7 +15853,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>France / Pays-Bas</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -15858,22 +15863,22 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Product Owner en full remote depuis la France, verifie ouvert par l'API Lever.</t>
+          <t>Poste senior sur plateforme coeur, full remote.</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/jobgether/5405e9ec-8ab3-4075-8f5e-96425e4f11a6</t>
+          <t>https://jobs.lever.co/jobgether/3efb5da5-0c07-4209-a4b6-037ead7571c2</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>75-90 K€</t>
+          <t>80-95 K€</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -15890,12 +15895,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>B2C Growth Product Manager</t>
+          <t>Senior Product Manager</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>n.c. (via Jobgether)</t>
+          <t>Pennylane</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -15910,156 +15915,166 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>Remote Europe</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Scale-up francaise, remote depuis n'importe ou en Europe. URL issue de WebSearch : l'API Lever n'a pas repondu sur ce slug, verifier que l'annonce est encore ouverte avant de candidater.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/pennylane/e821e150-f513-4297-86a7-6d2ee25ac50c</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>80-95 K€</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="69" t="inlineStr">
+        <is>
+          <t>⭐</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Hors profil</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Senior Product Manager - Core Platform (Remote)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Camunda</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>jobs.ashbyhq.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>Full remote</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Produit B2C oriente growth : recoupe directement WallOfTraders.com (acquisition SEO, paid social, boucle de retour utilisateurs).</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/jobgether/bae287fc-687d-48a6-a860-100430cbe25e</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>75-90 K€</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Ecarte : moteur Zeebe, systemes distribues, scalabilite et fiabilite ; expertise non couverte. Une seule candidature Camunda, celle sur Self Managed Service.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/camunda/b771e145-a5cf-4867-ad13-b54830e3b744</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>85-100 K€</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>14/08/2026</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="90" t="inlineStr">
-        <is>
-          <t>⭐⭐⭐</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Sr. Product Manager, Core Platform</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>n.c. (via Jobgether)</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>jobs.lever.co</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>France / Pays-Bas</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="69" t="inlineStr">
+        <is>
+          <t>⭐</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Hors profil</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Senior Product Builder - Connectors Experience - EMEA</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Camunda</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>jobs.ashbyhq.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>Full remote</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Poste senior sur plateforme coeur, full remote.</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/jobgether/3efb5da5-0c07-4209-a4b6-037ead7571c2</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Ecarte : annonce dupliquee par Camunda (version generique + version EMEA) et role de builder hands-on (prototype, build, ship, relecture de code). Une seule candidature Camunda, celle sur Self Managed Service.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/camunda/05cb2825-dcd9-40e6-bf92-bda409d99374</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>Resume_GaetanFRANCOIS_PM_Platform_EN.pdf</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>80-95 K€</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>14/08/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="90" t="inlineStr">
-        <is>
-          <t>⭐⭐⭐</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Senior Product Manager</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Pennylane</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>jobs.lever.co</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Europe</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Remote Europe</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Scale-up francaise, remote depuis n'importe ou en Europe. URL issue de WebSearch : l'API Lever n'a pas repondu sur ce slug, verifier que l'annonce est encore ouverte avant de candidater.</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/pennylane/e821e150-f513-4297-86a7-6d2ee25ac50c</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Resume_GaetanFRANCOIS_PM_EN.pdf</t>
-        </is>
-      </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>80-95 K€</t>
+          <t>85-100 K€</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">

</xml_diff>

<commit_message>
Camunda Self Managed: fourchettes salariales reelles de l'annonce et pretention relevee a 100-115 K€
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -15303,9 +15303,14 @@
           <t>Full remote</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Total Target Cash (base + variable) : US 143,8-231,9 K$ / UK 90,3-148,5 K£ / SG 178,6-267,9 KS$ / CA 152,7-251,2 KC$. Fourchette du mini marche Standard au maxi marche Major. Hors ces pays : embauche via Remote.com, calculateur personnalise apres le 1er entretien. VSOP (equity) en plus.</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Seule candidature Camunda retenue. Le poste porte sur l'installation, la configuration et l'exploitation de Camunda 8 chez le client (on-premises, configurations enterprise, reduction de la friction de deploiement, travail avec pre-sales et solution architects) ; c'est le parcours SAP HR on-prem vers SuccessFactors. Lacune a concéder en LM : Kubernetes et Helm.</t>
+          <t>Seule candidature Camunda retenue. Le poste porte sur l'installation, la configuration et l'exploitation de Camunda 8 chez le client (on-premises, configurations enterprise, reduction de la friction de deploiement, travail avec pre-sales et solution architects) ; c'est le parcours SAP HR on-prem vers SuccessFactors. Lacune a concéder en LM : Kubernetes et Helm. Salaire : viser 100-115 K€ TTC ; la France compte comme marche Standard, donc bas de fourchette des marches Standard (UK mini ~106 K€), et ils annoncent recruter dans la premiere moitie de la fourchette.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -15320,7 +15325,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>80-95 K€</t>
+          <t>100-115 K€</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">

</xml_diff>

<commit_message>
CV Ashby EN: variante deploiement client derivee du CV Constructor, ligne tableur mise a jour avec la grille salariale France
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/offres_emploi.xlsx
+++ b/offres_emploi.xlsx
@@ -1421,6 +1421,11 @@
           <t>Full remote</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>OTE 110-146 K€ (grille France) + equity</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>Encadrement d'une equipe de deploiement client sur l'EMEA, chez un editeur d'ATS. Quinze ans de deploiement SIRH multi-pays plus l'encadrement d'equipe : c'est le poste le plus proche du parcours reel dans cette relance. Full remote depuis l'Union europeenne.</t>
@@ -1433,12 +1438,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Resume_GaetanFRANCOIS_SIRH_EN.pdf</t>
+          <t>Resume_GaetanFRANCOIS_Ashby_EN.pdf</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>90-110 K€</t>
+          <t>110-146 K€ (OTE)</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">

</xml_diff>